<commit_message>
Added 3D Print Layout .3mf
</commit_message>
<xml_diff>
--- a/LC-CNC-BoM.xlsx
+++ b/LC-CNC-BoM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://liveutk.sharepoint.com/sites/UT_DesktopMillingMachine/Shared Documents/General/GitHub-Landon/LC-CNC/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1181" documentId="11_FCC9E17DDF51C54A1A3D9BFC69DB0C4BF401B41C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{03A9831F-5709-4459-843B-4295C5CE50DA}"/>
+  <xr:revisionPtr revIDLastSave="1183" documentId="11_FCC9E17DDF51C54A1A3D9BFC69DB0C4BF401B41C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1BDAAAB5-9E87-4D8C-88E8-9D5854070E70}"/>
   <bookViews>
-    <workbookView xWindow="1035" yWindow="1680" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1545" yWindow="1920" windowWidth="21600" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1777,6 +1777,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5552,6 +5556,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="fb0bfce0-b493-4733-b695-336371de64d4" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a816e368-bd7d-4e73-ae60-f7bbf4d187c7">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010049C730614A98FF4D948BAAFAA2763638" ma:contentTypeVersion="14" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="71752533c218a459f0bd7314a8d27046">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a816e368-bd7d-4e73-ae60-f7bbf4d187c7" xmlns:ns3="fb0bfce0-b493-4733-b695-336371de64d4" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="56df45e61c8cd6f396207a6803100ce0" ns2:_="" ns3:_="">
     <xsd:import namespace="a816e368-bd7d-4e73-ae60-f7bbf4d187c7"/>
@@ -5764,27 +5788,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2EA33EB9-975B-4CAF-BADE-D8C6854E172C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="fb0bfce0-b493-4733-b695-336371de64d4" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a816e368-bd7d-4e73-ae60-f7bbf4d187c7">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD534FFF-F9D4-45E9-B4A8-C5178968AA79}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="fb0bfce0-b493-4733-b695-336371de64d4"/>
+    <ds:schemaRef ds:uri="a816e368-bd7d-4e73-ae60-f7bbf4d187c7"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5B4CFA9-3BF7-4410-A240-4C3EA4FF6CE4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -5801,23 +5824,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2EA33EB9-975B-4CAF-BADE-D8C6854E172C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FD534FFF-F9D4-45E9-B4A8-C5178968AA79}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="fb0bfce0-b493-4733-b695-336371de64d4"/>
-    <ds:schemaRef ds:uri="a816e368-bd7d-4e73-ae60-f7bbf4d187c7"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>